<commit_message>
Runung the Bug resolve in Production Environment
</commit_message>
<xml_diff>
--- a/Upload Excel File/WhiteList Merchant Ip/WhiteList_MerchantIP.xlsx
+++ b/Upload Excel File/WhiteList Merchant Ip/WhiteList_MerchantIP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\Excel file\WhiteList Merchant Ip\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pg10-automation\Upload Excel File\WhiteList Merchant Ip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87D4B93-04D5-4672-9BB9-E965F4CAA47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6147CF60-22AD-461E-9DC0-2CEFE2EF79BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11175" xr2:uid="{EE0DE6B2-8B27-41C4-AEB0-1EC0728ED4FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EE0DE6B2-8B27-41C4-AEB0-1EC0728ED4FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>